<commit_message>
Updated calibration data (counts)
</commit_message>
<xml_diff>
--- a/data/calibration/counts.xlsx
+++ b/data/calibration/counts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vuhien/Desktop/Calibration/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA091AD8-0E16-F34F-88EA-0D8CA6F53789}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{342C7B1B-6EFA-FE46-A3A2-3BD6EF2F69C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="17320" xr2:uid="{F0941CDE-55DC-E949-AB0F-9CFF344905A0}"/>
   </bookViews>
@@ -1287,7 +1287,8 @@
         <v>51999999.999999993</v>
       </c>
       <c r="E20">
-        <v>0</v>
+        <f>3/(10^(-3)*0.01)</f>
+        <v>300000</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.2">
@@ -1306,7 +1307,8 @@
         <v>51999999.999999993</v>
       </c>
       <c r="E21">
-        <v>0</v>
+        <f>2/(10^(-3)*0.01)</f>
+        <v>199999.99999999997</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.2">
@@ -1325,7 +1327,8 @@
         <v>899999.99999999988</v>
       </c>
       <c r="E22">
-        <v>0</v>
+        <f>1/(10^(-3)*0.01)</f>
+        <v>99999.999999999985</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.2">
@@ -1344,7 +1347,8 @@
         <v>1599999.9999999998</v>
       </c>
       <c r="E23">
-        <v>0</v>
+        <f>2/(10^(-3)*0.01)</f>
+        <v>199999.99999999997</v>
       </c>
     </row>
   </sheetData>

</xml_diff>